<commit_message>
added new data source
</commit_message>
<xml_diff>
--- a/20250426_Vipers/01_source/Barges and Zones.xlsx
+++ b/20250426_Vipers/01_source/Barges and Zones.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25831"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://usaf-my.dps.mil/personal/jennifer_shelton_4_us_af_mil/Documents/Desktop/Barge Status/sample files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Professional\04_Git\AI_Power_Studio\20250426_Vipers\01_source\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{31585970-6A4D-4777-BD14-7E9A9FFB7C7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA0A4863-6C48-4448-B852-B3A2568BFE8A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5775" yWindow="1275" windowWidth="21150" windowHeight="11145" xr2:uid="{81B4CA33-04E4-4F2F-A71F-A37A32AC4D53}"/>
+    <workbookView xWindow="4670" yWindow="430" windowWidth="31320" windowHeight="20370" activeTab="1" xr2:uid="{81B4CA33-04E4-4F2F-A71F-A37A32AC4D53}"/>
   </bookViews>
   <sheets>
     <sheet name="Barges &amp; Zones" sheetId="2" r:id="rId1"/>
+    <sheet name="Barges" sheetId="3" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Barges &amp; Zones'!$A$1:$E$1</definedName>
@@ -23,23 +24,12 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="74">
   <si>
     <t>C</t>
   </si>
@@ -240,18 +230,46 @@
   </si>
   <si>
     <t>ACC</t>
+  </si>
+  <si>
+    <t>Barge 1</t>
+  </si>
+  <si>
+    <t>Barge 2</t>
+  </si>
+  <si>
+    <t>Barge 3</t>
+  </si>
+  <si>
+    <t>Barge 4</t>
+  </si>
+  <si>
+    <t>Barge 5</t>
+  </si>
+  <si>
+    <t>Barge 6</t>
+  </si>
+  <si>
+    <t>MISC</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
+      <name val="等线"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -283,7 +301,7 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="常规" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="2">
     <dxf>
@@ -317,7 +335,7 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 主题​​">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -327,39 +345,39 @@
         <a:sysClr val="window" lastClr="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="44546A"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="E7E6E6"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="156082"/>
+        <a:srgbClr val="4472C4"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="ED7D31"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="A5A5A5"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="FFC000"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="5B9BD5"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="70AD47"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="467886"/>
+        <a:srgbClr val="0563C1"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -411,7 +429,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Calibri" panose="020F0502020204030204"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -522,6 +540,13 @@
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
+        <a:ln w="6350" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+          <a:miter lim="800000"/>
+        </a:ln>
         <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
@@ -530,13 +555,6 @@
           <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
@@ -601,31 +619,11 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -634,14 +632,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C307BC7E-CB43-4954-8889-992254CA448F}">
   <dimension ref="A1:G55"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.140625" style="2"/>
-    <col min="5" max="5" width="9.140625" style="1"/>
-    <col min="8" max="13" width="9.5703125" customWidth="1"/>
+    <col min="1" max="1" width="9.1640625" style="2"/>
+    <col min="5" max="5" width="9.1640625" style="1"/>
+    <col min="8" max="13" width="9.58203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>66</v>
       </c>
@@ -655,12 +653,12 @@
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>62</v>
       </c>
       <c r="B2" t="str">
-        <f>IF($A2="651","Barge1",IF($A2="101","Barge1",IF(A2="201","Barge 1",IF(A2="801","Barge 2",IF($A2="351", "Barge 2", IF($A2="151", "Barge 3",IF($A2="251","Barge 3",IF($A2="451", "Barge 4",IF($A2="551", "Barge 4",IF($A2="301","Barge 5",IF($A2="401","Barge 5",IF($A2="501","Barge 6",IF($A2="851","Barge 6",IF($A2="601","Barge 6",IF($A2="VC651","Barge1",IF($A2="VC101","Barge1",IF(A2="VC201","Barge 1",IF(A2="VC801","Barge 2",IF($A2="VC351", "Barge 2", IF($A2="VC151", "Barge 3",IF($A2="VC251","Barge 3",IF($A2="VC451", "Barge 4",IF($A2="VC551", "Barge 4",IF($A2="VC301","Barge 5",IF($A2="VC401","Barge 5",IF($A2="VC501","Barge 6",IF($A2="VC851","Barge 6",IF($A2="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" ref="B2:B33" si="0">IF($A2="651","Barge1",IF($A2="101","Barge1",IF(A2="201","Barge 1",IF(A2="801","Barge 2",IF($A2="351", "Barge 2", IF($A2="151", "Barge 3",IF($A2="251","Barge 3",IF($A2="451", "Barge 4",IF($A2="551", "Barge 4",IF($A2="301","Barge 5",IF($A2="401","Barge 5",IF($A2="501","Barge 6",IF($A2="851","Barge 6",IF($A2="601","Barge 6",IF($A2="VC651","Barge1",IF($A2="VC101","Barge1",IF(A2="VC201","Barge 1",IF(A2="VC801","Barge 2",IF($A2="VC351", "Barge 2", IF($A2="VC151", "Barge 3",IF($A2="VC251","Barge 3",IF($A2="VC451", "Barge 4",IF($A2="VC551", "Barge 4",IF($A2="VC301","Barge 5",IF($A2="VC401","Barge 5",IF($A2="VC501","Barge 6",IF($A2="VC851","Barge 6",IF($A2="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
         <v>Barge 1</v>
       </c>
       <c r="C2" t="s">
@@ -670,12 +668,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>61</v>
       </c>
       <c r="B3" t="str">
-        <f>IF($A3="651","Barge1",IF($A3="101","Barge1",IF(A3="201","Barge 1",IF(A3="801","Barge 2",IF($A3="351", "Barge 2", IF($A3="151", "Barge 3",IF($A3="251","Barge 3",IF($A3="451", "Barge 4",IF($A3="551", "Barge 4",IF($A3="301","Barge 5",IF($A3="401","Barge 5",IF($A3="501","Barge 6",IF($A3="851","Barge 6",IF($A3="601","Barge 6",IF($A3="VC651","Barge1",IF($A3="VC101","Barge1",IF(A3="VC201","Barge 1",IF(A3="VC801","Barge 2",IF($A3="VC351", "Barge 2", IF($A3="VC151", "Barge 3",IF($A3="VC251","Barge 3",IF($A3="VC451", "Barge 4",IF($A3="VC551", "Barge 4",IF($A3="VC301","Barge 5",IF($A3="VC401","Barge 5",IF($A3="VC501","Barge 6",IF($A3="VC851","Barge 6",IF($A3="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 1</v>
       </c>
       <c r="C3" t="s">
@@ -685,12 +683,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>60</v>
       </c>
       <c r="B4" t="str">
-        <f>IF($A4="651","Barge1",IF($A4="101","Barge1",IF(A4="201","Barge 1",IF(A4="801","Barge 2",IF($A4="351", "Barge 2", IF($A4="151", "Barge 3",IF($A4="251","Barge 3",IF($A4="451", "Barge 4",IF($A4="551", "Barge 4",IF($A4="301","Barge 5",IF($A4="401","Barge 5",IF($A4="501","Barge 6",IF($A4="851","Barge 6",IF($A4="601","Barge 6",IF($A4="VC651","Barge1",IF($A4="VC101","Barge1",IF(A4="VC201","Barge 1",IF(A4="VC801","Barge 2",IF($A4="VC351", "Barge 2", IF($A4="VC151", "Barge 3",IF($A4="VC251","Barge 3",IF($A4="VC451", "Barge 4",IF($A4="VC551", "Barge 4",IF($A4="VC301","Barge 5",IF($A4="VC401","Barge 5",IF($A4="VC501","Barge 6",IF($A4="VC851","Barge 6",IF($A4="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 2</v>
       </c>
       <c r="C4" t="s">
@@ -700,12 +698,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>59</v>
       </c>
       <c r="B5" t="str">
-        <f>IF($A5="651","Barge1",IF($A5="101","Barge1",IF(A5="201","Barge 1",IF(A5="801","Barge 2",IF($A5="351", "Barge 2", IF($A5="151", "Barge 3",IF($A5="251","Barge 3",IF($A5="451", "Barge 4",IF($A5="551", "Barge 4",IF($A5="301","Barge 5",IF($A5="401","Barge 5",IF($A5="501","Barge 6",IF($A5="851","Barge 6",IF($A5="601","Barge 6",IF($A5="VC651","Barge1",IF($A5="VC101","Barge1",IF(A5="VC201","Barge 1",IF(A5="VC801","Barge 2",IF($A5="VC351", "Barge 2", IF($A5="VC151", "Barge 3",IF($A5="VC251","Barge 3",IF($A5="VC451", "Barge 4",IF($A5="VC551", "Barge 4",IF($A5="VC301","Barge 5",IF($A5="VC401","Barge 5",IF($A5="VC501","Barge 6",IF($A5="VC851","Barge 6",IF($A5="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 2</v>
       </c>
       <c r="C5" t="s">
@@ -715,12 +713,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>58</v>
       </c>
       <c r="B6" t="str">
-        <f>IF($A6="651","Barge1",IF($A6="101","Barge1",IF(A6="201","Barge 1",IF(A6="801","Barge 2",IF($A6="351", "Barge 2", IF($A6="151", "Barge 3",IF($A6="251","Barge 3",IF($A6="451", "Barge 4",IF($A6="551", "Barge 4",IF($A6="301","Barge 5",IF($A6="401","Barge 5",IF($A6="501","Barge 6",IF($A6="851","Barge 6",IF($A6="601","Barge 6",IF($A6="VC651","Barge1",IF($A6="VC101","Barge1",IF(A6="VC201","Barge 1",IF(A6="VC801","Barge 2",IF($A6="VC351", "Barge 2", IF($A6="VC151", "Barge 3",IF($A6="VC251","Barge 3",IF($A6="VC451", "Barge 4",IF($A6="VC551", "Barge 4",IF($A6="VC301","Barge 5",IF($A6="VC401","Barge 5",IF($A6="VC501","Barge 6",IF($A6="VC851","Barge 6",IF($A6="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 2</v>
       </c>
       <c r="C6" t="s">
@@ -730,12 +728,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>57</v>
       </c>
       <c r="B7" t="str">
-        <f>IF($A7="651","Barge1",IF($A7="101","Barge1",IF(A7="201","Barge 1",IF(A7="801","Barge 2",IF($A7="351", "Barge 2", IF($A7="151", "Barge 3",IF($A7="251","Barge 3",IF($A7="451", "Barge 4",IF($A7="551", "Barge 4",IF($A7="301","Barge 5",IF($A7="401","Barge 5",IF($A7="501","Barge 6",IF($A7="851","Barge 6",IF($A7="601","Barge 6",IF($A7="VC651","Barge1",IF($A7="VC101","Barge1",IF(A7="VC201","Barge 1",IF(A7="VC801","Barge 2",IF($A7="VC351", "Barge 2", IF($A7="VC151", "Barge 3",IF($A7="VC251","Barge 3",IF($A7="VC451", "Barge 4",IF($A7="VC551", "Barge 4",IF($A7="VC301","Barge 5",IF($A7="VC401","Barge 5",IF($A7="VC501","Barge 6",IF($A7="VC851","Barge 6",IF($A7="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 2</v>
       </c>
       <c r="C7" t="s">
@@ -745,12 +743,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>55</v>
       </c>
       <c r="B8" t="str">
-        <f>IF($A8="651","Barge1",IF($A8="101","Barge1",IF(A8="201","Barge 1",IF(A8="801","Barge 2",IF($A8="351", "Barge 2", IF($A8="151", "Barge 3",IF($A8="251","Barge 3",IF($A8="451", "Barge 4",IF($A8="551", "Barge 4",IF($A8="301","Barge 5",IF($A8="401","Barge 5",IF($A8="501","Barge 6",IF($A8="851","Barge 6",IF($A8="601","Barge 6",IF($A8="VC651","Barge1",IF($A8="VC101","Barge1",IF(A8="VC201","Barge 1",IF(A8="VC801","Barge 2",IF($A8="VC351", "Barge 2", IF($A8="VC151", "Barge 3",IF($A8="VC251","Barge 3",IF($A8="VC451", "Barge 4",IF($A8="VC551", "Barge 4",IF($A8="VC301","Barge 5",IF($A8="VC401","Barge 5",IF($A8="VC501","Barge 6",IF($A8="VC851","Barge 6",IF($A8="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 3</v>
       </c>
       <c r="C8" t="s">
@@ -760,12 +758,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>54</v>
       </c>
       <c r="B9" t="str">
-        <f>IF($A9="651","Barge1",IF($A9="101","Barge1",IF(A9="201","Barge 1",IF(A9="801","Barge 2",IF($A9="351", "Barge 2", IF($A9="151", "Barge 3",IF($A9="251","Barge 3",IF($A9="451", "Barge 4",IF($A9="551", "Barge 4",IF($A9="301","Barge 5",IF($A9="401","Barge 5",IF($A9="501","Barge 6",IF($A9="851","Barge 6",IF($A9="601","Barge 6",IF($A9="VC651","Barge1",IF($A9="VC101","Barge1",IF(A9="VC201","Barge 1",IF(A9="VC801","Barge 2",IF($A9="VC351", "Barge 2", IF($A9="VC151", "Barge 3",IF($A9="VC251","Barge 3",IF($A9="VC451", "Barge 4",IF($A9="VC551", "Barge 4",IF($A9="VC301","Barge 5",IF($A9="VC401","Barge 5",IF($A9="VC501","Barge 6",IF($A9="VC851","Barge 6",IF($A9="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 3</v>
       </c>
       <c r="C9" t="s">
@@ -776,12 +774,12 @@
       </c>
       <c r="G9" s="1"/>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>53</v>
       </c>
       <c r="B10" t="str">
-        <f>IF($A10="651","Barge1",IF($A10="101","Barge1",IF(A10="201","Barge 1",IF(A10="801","Barge 2",IF($A10="351", "Barge 2", IF($A10="151", "Barge 3",IF($A10="251","Barge 3",IF($A10="451", "Barge 4",IF($A10="551", "Barge 4",IF($A10="301","Barge 5",IF($A10="401","Barge 5",IF($A10="501","Barge 6",IF($A10="851","Barge 6",IF($A10="601","Barge 6",IF($A10="VC651","Barge1",IF($A10="VC101","Barge1",IF(A10="VC201","Barge 1",IF(A10="VC801","Barge 2",IF($A10="VC351", "Barge 2", IF($A10="VC151", "Barge 3",IF($A10="VC251","Barge 3",IF($A10="VC451", "Barge 4",IF($A10="VC551", "Barge 4",IF($A10="VC301","Barge 5",IF($A10="VC401","Barge 5",IF($A10="VC501","Barge 6",IF($A10="VC851","Barge 6",IF($A10="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 3</v>
       </c>
       <c r="C10" t="s">
@@ -792,12 +790,12 @@
       </c>
       <c r="G10" s="1"/>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>52</v>
       </c>
       <c r="B11" t="str">
-        <f>IF($A11="651","Barge1",IF($A11="101","Barge1",IF(A11="201","Barge 1",IF(A11="801","Barge 2",IF($A11="351", "Barge 2", IF($A11="151", "Barge 3",IF($A11="251","Barge 3",IF($A11="451", "Barge 4",IF($A11="551", "Barge 4",IF($A11="301","Barge 5",IF($A11="401","Barge 5",IF($A11="501","Barge 6",IF($A11="851","Barge 6",IF($A11="601","Barge 6",IF($A11="VC651","Barge1",IF($A11="VC101","Barge1",IF(A11="VC201","Barge 1",IF(A11="VC801","Barge 2",IF($A11="VC351", "Barge 2", IF($A11="VC151", "Barge 3",IF($A11="VC251","Barge 3",IF($A11="VC451", "Barge 4",IF($A11="VC551", "Barge 4",IF($A11="VC301","Barge 5",IF($A11="VC401","Barge 5",IF($A11="VC501","Barge 6",IF($A11="VC851","Barge 6",IF($A11="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 3</v>
       </c>
       <c r="C11" t="s">
@@ -808,12 +806,12 @@
       </c>
       <c r="G11" s="1"/>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>50</v>
       </c>
       <c r="B12" t="str">
-        <f>IF($A12="651","Barge1",IF($A12="101","Barge1",IF(A12="201","Barge 1",IF(A12="801","Barge 2",IF($A12="351", "Barge 2", IF($A12="151", "Barge 3",IF($A12="251","Barge 3",IF($A12="451", "Barge 4",IF($A12="551", "Barge 4",IF($A12="301","Barge 5",IF($A12="401","Barge 5",IF($A12="501","Barge 6",IF($A12="851","Barge 6",IF($A12="601","Barge 6",IF($A12="VC651","Barge1",IF($A12="VC101","Barge1",IF(A12="VC201","Barge 1",IF(A12="VC801","Barge 2",IF($A12="VC351", "Barge 2", IF($A12="VC151", "Barge 3",IF($A12="VC251","Barge 3",IF($A12="VC451", "Barge 4",IF($A12="VC551", "Barge 4",IF($A12="VC301","Barge 5",IF($A12="VC401","Barge 5",IF($A12="VC501","Barge 6",IF($A12="VC851","Barge 6",IF($A12="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 4</v>
       </c>
       <c r="C12" t="s">
@@ -824,12 +822,12 @@
       </c>
       <c r="G12" s="1"/>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>49</v>
       </c>
       <c r="B13" t="str">
-        <f>IF($A13="651","Barge1",IF($A13="101","Barge1",IF(A13="201","Barge 1",IF(A13="801","Barge 2",IF($A13="351", "Barge 2", IF($A13="151", "Barge 3",IF($A13="251","Barge 3",IF($A13="451", "Barge 4",IF($A13="551", "Barge 4",IF($A13="301","Barge 5",IF($A13="401","Barge 5",IF($A13="501","Barge 6",IF($A13="851","Barge 6",IF($A13="601","Barge 6",IF($A13="VC651","Barge1",IF($A13="VC101","Barge1",IF(A13="VC201","Barge 1",IF(A13="VC801","Barge 2",IF($A13="VC351", "Barge 2", IF($A13="VC151", "Barge 3",IF($A13="VC251","Barge 3",IF($A13="VC451", "Barge 4",IF($A13="VC551", "Barge 4",IF($A13="VC301","Barge 5",IF($A13="VC401","Barge 5",IF($A13="VC501","Barge 6",IF($A13="VC851","Barge 6",IF($A13="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 4</v>
       </c>
       <c r="C13" t="s">
@@ -840,12 +838,12 @@
       </c>
       <c r="G13" s="1"/>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>48</v>
       </c>
       <c r="B14" t="str">
-        <f>IF($A14="651","Barge1",IF($A14="101","Barge1",IF(A14="201","Barge 1",IF(A14="801","Barge 2",IF($A14="351", "Barge 2", IF($A14="151", "Barge 3",IF($A14="251","Barge 3",IF($A14="451", "Barge 4",IF($A14="551", "Barge 4",IF($A14="301","Barge 5",IF($A14="401","Barge 5",IF($A14="501","Barge 6",IF($A14="851","Barge 6",IF($A14="601","Barge 6",IF($A14="VC651","Barge1",IF($A14="VC101","Barge1",IF(A14="VC201","Barge 1",IF(A14="VC801","Barge 2",IF($A14="VC351", "Barge 2", IF($A14="VC151", "Barge 3",IF($A14="VC251","Barge 3",IF($A14="VC451", "Barge 4",IF($A14="VC551", "Barge 4",IF($A14="VC301","Barge 5",IF($A14="VC401","Barge 5",IF($A14="VC501","Barge 6",IF($A14="VC851","Barge 6",IF($A14="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 4</v>
       </c>
       <c r="C14" t="s">
@@ -856,12 +854,12 @@
       </c>
       <c r="G14" s="1"/>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>47</v>
       </c>
       <c r="B15" t="str">
-        <f>IF($A15="651","Barge1",IF($A15="101","Barge1",IF(A15="201","Barge 1",IF(A15="801","Barge 2",IF($A15="351", "Barge 2", IF($A15="151", "Barge 3",IF($A15="251","Barge 3",IF($A15="451", "Barge 4",IF($A15="551", "Barge 4",IF($A15="301","Barge 5",IF($A15="401","Barge 5",IF($A15="501","Barge 6",IF($A15="851","Barge 6",IF($A15="601","Barge 6",IF($A15="VC651","Barge1",IF($A15="VC101","Barge1",IF(A15="VC201","Barge 1",IF(A15="VC801","Barge 2",IF($A15="VC351", "Barge 2", IF($A15="VC151", "Barge 3",IF($A15="VC251","Barge 3",IF($A15="VC451", "Barge 4",IF($A15="VC551", "Barge 4",IF($A15="VC301","Barge 5",IF($A15="VC401","Barge 5",IF($A15="VC501","Barge 6",IF($A15="VC851","Barge 6",IF($A15="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 4</v>
       </c>
       <c r="C15" t="s">
@@ -872,12 +870,12 @@
       </c>
       <c r="G15" s="1"/>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>45</v>
       </c>
       <c r="B16" t="str">
-        <f>IF($A16="651","Barge1",IF($A16="101","Barge1",IF(A16="201","Barge 1",IF(A16="801","Barge 2",IF($A16="351", "Barge 2", IF($A16="151", "Barge 3",IF($A16="251","Barge 3",IF($A16="451", "Barge 4",IF($A16="551", "Barge 4",IF($A16="301","Barge 5",IF($A16="401","Barge 5",IF($A16="501","Barge 6",IF($A16="851","Barge 6",IF($A16="601","Barge 6",IF($A16="VC651","Barge1",IF($A16="VC101","Barge1",IF(A16="VC201","Barge 1",IF(A16="VC801","Barge 2",IF($A16="VC351", "Barge 2", IF($A16="VC151", "Barge 3",IF($A16="VC251","Barge 3",IF($A16="VC451", "Barge 4",IF($A16="VC551", "Barge 4",IF($A16="VC301","Barge 5",IF($A16="VC401","Barge 5",IF($A16="VC501","Barge 6",IF($A16="VC851","Barge 6",IF($A16="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 5</v>
       </c>
       <c r="C16" t="s">
@@ -888,12 +886,12 @@
       </c>
       <c r="G16" s="1"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>44</v>
       </c>
       <c r="B17" t="str">
-        <f>IF($A17="651","Barge1",IF($A17="101","Barge1",IF(A17="201","Barge 1",IF(A17="801","Barge 2",IF($A17="351", "Barge 2", IF($A17="151", "Barge 3",IF($A17="251","Barge 3",IF($A17="451", "Barge 4",IF($A17="551", "Barge 4",IF($A17="301","Barge 5",IF($A17="401","Barge 5",IF($A17="501","Barge 6",IF($A17="851","Barge 6",IF($A17="601","Barge 6",IF($A17="VC651","Barge1",IF($A17="VC101","Barge1",IF(A17="VC201","Barge 1",IF(A17="VC801","Barge 2",IF($A17="VC351", "Barge 2", IF($A17="VC151", "Barge 3",IF($A17="VC251","Barge 3",IF($A17="VC451", "Barge 4",IF($A17="VC551", "Barge 4",IF($A17="VC301","Barge 5",IF($A17="VC401","Barge 5",IF($A17="VC501","Barge 6",IF($A17="VC851","Barge 6",IF($A17="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 5</v>
       </c>
       <c r="C17" t="s">
@@ -903,12 +901,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>43</v>
       </c>
       <c r="B18" t="str">
-        <f>IF($A18="651","Barge1",IF($A18="101","Barge1",IF(A18="201","Barge 1",IF(A18="801","Barge 2",IF($A18="351", "Barge 2", IF($A18="151", "Barge 3",IF($A18="251","Barge 3",IF($A18="451", "Barge 4",IF($A18="551", "Barge 4",IF($A18="301","Barge 5",IF($A18="401","Barge 5",IF($A18="501","Barge 6",IF($A18="851","Barge 6",IF($A18="601","Barge 6",IF($A18="VC651","Barge1",IF($A18="VC101","Barge1",IF(A18="VC201","Barge 1",IF(A18="VC801","Barge 2",IF($A18="VC351", "Barge 2", IF($A18="VC151", "Barge 3",IF($A18="VC251","Barge 3",IF($A18="VC451", "Barge 4",IF($A18="VC551", "Barge 4",IF($A18="VC301","Barge 5",IF($A18="VC401","Barge 5",IF($A18="VC501","Barge 6",IF($A18="VC851","Barge 6",IF($A18="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 5</v>
       </c>
       <c r="C18" t="s">
@@ -918,12 +916,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>42</v>
       </c>
       <c r="B19" t="str">
-        <f>IF($A19="651","Barge1",IF($A19="101","Barge1",IF(A19="201","Barge 1",IF(A19="801","Barge 2",IF($A19="351", "Barge 2", IF($A19="151", "Barge 3",IF($A19="251","Barge 3",IF($A19="451", "Barge 4",IF($A19="551", "Barge 4",IF($A19="301","Barge 5",IF($A19="401","Barge 5",IF($A19="501","Barge 6",IF($A19="851","Barge 6",IF($A19="601","Barge 6",IF($A19="VC651","Barge1",IF($A19="VC101","Barge1",IF(A19="VC201","Barge 1",IF(A19="VC801","Barge 2",IF($A19="VC351", "Barge 2", IF($A19="VC151", "Barge 3",IF($A19="VC251","Barge 3",IF($A19="VC451", "Barge 4",IF($A19="VC551", "Barge 4",IF($A19="VC301","Barge 5",IF($A19="VC401","Barge 5",IF($A19="VC501","Barge 6",IF($A19="VC851","Barge 6",IF($A19="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 5</v>
       </c>
       <c r="C19" t="s">
@@ -933,12 +931,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>40</v>
       </c>
       <c r="B20" t="str">
-        <f>IF($A20="651","Barge1",IF($A20="101","Barge1",IF(A20="201","Barge 1",IF(A20="801","Barge 2",IF($A20="351", "Barge 2", IF($A20="151", "Barge 3",IF($A20="251","Barge 3",IF($A20="451", "Barge 4",IF($A20="551", "Barge 4",IF($A20="301","Barge 5",IF($A20="401","Barge 5",IF($A20="501","Barge 6",IF($A20="851","Barge 6",IF($A20="601","Barge 6",IF($A20="VC651","Barge1",IF($A20="VC101","Barge1",IF(A20="VC201","Barge 1",IF(A20="VC801","Barge 2",IF($A20="VC351", "Barge 2", IF($A20="VC151", "Barge 3",IF($A20="VC251","Barge 3",IF($A20="VC451", "Barge 4",IF($A20="VC551", "Barge 4",IF($A20="VC301","Barge 5",IF($A20="VC401","Barge 5",IF($A20="VC501","Barge 6",IF($A20="VC851","Barge 6",IF($A20="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 6</v>
       </c>
       <c r="C20" t="s">
@@ -948,12 +946,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B21" t="str">
-        <f>IF($A21="651","Barge1",IF($A21="101","Barge1",IF(A21="201","Barge 1",IF(A21="801","Barge 2",IF($A21="351", "Barge 2", IF($A21="151", "Barge 3",IF($A21="251","Barge 3",IF($A21="451", "Barge 4",IF($A21="551", "Barge 4",IF($A21="301","Barge 5",IF($A21="401","Barge 5",IF($A21="501","Barge 6",IF($A21="851","Barge 6",IF($A21="601","Barge 6",IF($A21="VC651","Barge1",IF($A21="VC101","Barge1",IF(A21="VC201","Barge 1",IF(A21="VC801","Barge 2",IF($A21="VC351", "Barge 2", IF($A21="VC151", "Barge 3",IF($A21="VC251","Barge 3",IF($A21="VC451", "Barge 4",IF($A21="VC551", "Barge 4",IF($A21="VC301","Barge 5",IF($A21="VC401","Barge 5",IF($A21="VC501","Barge 6",IF($A21="VC851","Barge 6",IF($A21="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 6</v>
       </c>
       <c r="C21" t="s">
@@ -963,12 +961,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>38</v>
       </c>
       <c r="B22" t="str">
-        <f>IF($A22="651","Barge1",IF($A22="101","Barge1",IF(A22="201","Barge 1",IF(A22="801","Barge 2",IF($A22="351", "Barge 2", IF($A22="151", "Barge 3",IF($A22="251","Barge 3",IF($A22="451", "Barge 4",IF($A22="551", "Barge 4",IF($A22="301","Barge 5",IF($A22="401","Barge 5",IF($A22="501","Barge 6",IF($A22="851","Barge 6",IF($A22="601","Barge 6",IF($A22="VC651","Barge1",IF($A22="VC101","Barge1",IF(A22="VC201","Barge 1",IF(A22="VC801","Barge 2",IF($A22="VC351", "Barge 2", IF($A22="VC151", "Barge 3",IF($A22="VC251","Barge 3",IF($A22="VC451", "Barge 4",IF($A22="VC551", "Barge 4",IF($A22="VC301","Barge 5",IF($A22="VC401","Barge 5",IF($A22="VC501","Barge 6",IF($A22="VC851","Barge 6",IF($A22="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 6</v>
       </c>
       <c r="C22" t="s">
@@ -978,12 +976,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>37</v>
       </c>
       <c r="B23" t="str">
-        <f>IF($A23="651","Barge1",IF($A23="101","Barge1",IF(A23="201","Barge 1",IF(A23="801","Barge 2",IF($A23="351", "Barge 2", IF($A23="151", "Barge 3",IF($A23="251","Barge 3",IF($A23="451", "Barge 4",IF($A23="551", "Barge 4",IF($A23="301","Barge 5",IF($A23="401","Barge 5",IF($A23="501","Barge 6",IF($A23="851","Barge 6",IF($A23="601","Barge 6",IF($A23="VC651","Barge1",IF($A23="VC101","Barge1",IF(A23="VC201","Barge 1",IF(A23="VC801","Barge 2",IF($A23="VC351", "Barge 2", IF($A23="VC151", "Barge 3",IF($A23="VC251","Barge 3",IF($A23="VC451", "Barge 4",IF($A23="VC551", "Barge 4",IF($A23="VC301","Barge 5",IF($A23="VC401","Barge 5",IF($A23="VC501","Barge 6",IF($A23="VC851","Barge 6",IF($A23="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 6</v>
       </c>
       <c r="C23" t="s">
@@ -993,12 +991,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>36</v>
       </c>
       <c r="B24" t="str">
-        <f>IF($A24="651","Barge1",IF($A24="101","Barge1",IF(A24="201","Barge 1",IF(A24="801","Barge 2",IF($A24="351", "Barge 2", IF($A24="151", "Barge 3",IF($A24="251","Barge 3",IF($A24="451", "Barge 4",IF($A24="551", "Barge 4",IF($A24="301","Barge 5",IF($A24="401","Barge 5",IF($A24="501","Barge 6",IF($A24="851","Barge 6",IF($A24="601","Barge 6",IF($A24="VC651","Barge1",IF($A24="VC101","Barge1",IF(A24="VC201","Barge 1",IF(A24="VC801","Barge 2",IF($A24="VC351", "Barge 2", IF($A24="VC151", "Barge 3",IF($A24="VC251","Barge 3",IF($A24="VC451", "Barge 4",IF($A24="VC551", "Barge 4",IF($A24="VC301","Barge 5",IF($A24="VC401","Barge 5",IF($A24="VC501","Barge 6",IF($A24="VC851","Barge 6",IF($A24="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge 6</v>
       </c>
       <c r="C24" t="s">
@@ -1008,12 +1006,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>34</v>
       </c>
       <c r="B25" t="str">
-        <f>IF($A25="651","Barge1",IF($A25="101","Barge1",IF(A25="201","Barge 1",IF(A25="801","Barge 2",IF($A25="351", "Barge 2", IF($A25="151", "Barge 3",IF($A25="251","Barge 3",IF($A25="451", "Barge 4",IF($A25="551", "Barge 4",IF($A25="301","Barge 5",IF($A25="401","Barge 5",IF($A25="501","Barge 6",IF($A25="851","Barge 6",IF($A25="601","Barge 6",IF($A25="VC651","Barge1",IF($A25="VC101","Barge1",IF(A25="VC201","Barge 1",IF(A25="VC801","Barge 2",IF($A25="VC351", "Barge 2", IF($A25="VC151", "Barge 3",IF($A25="VC251","Barge 3",IF($A25="VC451", "Barge 4",IF($A25="VC551", "Barge 4",IF($A25="VC301","Barge 5",IF($A25="VC401","Barge 5",IF($A25="VC501","Barge 6",IF($A25="VC851","Barge 6",IF($A25="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge1</v>
       </c>
       <c r="C25" t="s">
@@ -1023,12 +1021,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B26" t="str">
-        <f>IF($A26="651","Barge1",IF($A26="101","Barge1",IF(A26="201","Barge 1",IF(A26="801","Barge 2",IF($A26="351", "Barge 2", IF($A26="151", "Barge 3",IF($A26="251","Barge 3",IF($A26="451", "Barge 4",IF($A26="551", "Barge 4",IF($A26="301","Barge 5",IF($A26="401","Barge 5",IF($A26="501","Barge 6",IF($A26="851","Barge 6",IF($A26="601","Barge 6",IF($A26="VC651","Barge1",IF($A26="VC101","Barge1",IF(A26="VC201","Barge 1",IF(A26="VC801","Barge 2",IF($A26="VC351", "Barge 2", IF($A26="VC151", "Barge 3",IF($A26="VC251","Barge 3",IF($A26="VC451", "Barge 4",IF($A26="VC551", "Barge 4",IF($A26="VC301","Barge 5",IF($A26="VC401","Barge 5",IF($A26="VC501","Barge 6",IF($A26="VC851","Barge 6",IF($A26="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge1</v>
       </c>
       <c r="C26" t="s">
@@ -1038,12 +1036,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>32</v>
       </c>
       <c r="B27" t="str">
-        <f>IF($A27="651","Barge1",IF($A27="101","Barge1",IF(A27="201","Barge 1",IF(A27="801","Barge 2",IF($A27="351", "Barge 2", IF($A27="151", "Barge 3",IF($A27="251","Barge 3",IF($A27="451", "Barge 4",IF($A27="551", "Barge 4",IF($A27="301","Barge 5",IF($A27="401","Barge 5",IF($A27="501","Barge 6",IF($A27="851","Barge 6",IF($A27="601","Barge 6",IF($A27="VC651","Barge1",IF($A27="VC101","Barge1",IF(A27="VC201","Barge 1",IF(A27="VC801","Barge 2",IF($A27="VC351", "Barge 2", IF($A27="VC151", "Barge 3",IF($A27="VC251","Barge 3",IF($A27="VC451", "Barge 4",IF($A27="VC551", "Barge 4",IF($A27="VC301","Barge 5",IF($A27="VC401","Barge 5",IF($A27="VC501","Barge 6",IF($A27="VC851","Barge 6",IF($A27="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>Barge1</v>
       </c>
       <c r="C27" t="s">
@@ -1053,12 +1051,12 @@
         <v>30</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>29</v>
       </c>
       <c r="B28" t="str">
-        <f>IF($A28="651","Barge1",IF($A28="101","Barge1",IF(A28="201","Barge 1",IF(A28="801","Barge 2",IF($A28="351", "Barge 2", IF($A28="151", "Barge 3",IF($A28="251","Barge 3",IF($A28="451", "Barge 4",IF($A28="551", "Barge 4",IF($A28="301","Barge 5",IF($A28="401","Barge 5",IF($A28="501","Barge 6",IF($A28="851","Barge 6",IF($A28="601","Barge 6",IF($A28="VC651","Barge1",IF($A28="VC101","Barge1",IF(A28="VC201","Barge 1",IF(A28="VC801","Barge 2",IF($A28="VC351", "Barge 2", IF($A28="VC151", "Barge 3",IF($A28="VC251","Barge 3",IF($A28="VC451", "Barge 4",IF($A28="VC551", "Barge 4",IF($A28="VC301","Barge 5",IF($A28="VC401","Barge 5",IF($A28="VC501","Barge 6",IF($A28="VC851","Barge 6",IF($A28="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>MISC</v>
       </c>
       <c r="C28" t="s">
@@ -1068,12 +1066,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>28</v>
       </c>
       <c r="B29" t="str">
-        <f>IF($A29="651","Barge1",IF($A29="101","Barge1",IF(A29="201","Barge 1",IF(A29="801","Barge 2",IF($A29="351", "Barge 2", IF($A29="151", "Barge 3",IF($A29="251","Barge 3",IF($A29="451", "Barge 4",IF($A29="551", "Barge 4",IF($A29="301","Barge 5",IF($A29="401","Barge 5",IF($A29="501","Barge 6",IF($A29="851","Barge 6",IF($A29="601","Barge 6",IF($A29="VC651","Barge1",IF($A29="VC101","Barge1",IF(A29="VC201","Barge 1",IF(A29="VC801","Barge 2",IF($A29="VC351", "Barge 2", IF($A29="VC151", "Barge 3",IF($A29="VC251","Barge 3",IF($A29="VC451", "Barge 4",IF($A29="VC551", "Barge 4",IF($A29="VC301","Barge 5",IF($A29="VC401","Barge 5",IF($A29="VC501","Barge 6",IF($A29="VC851","Barge 6",IF($A29="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>MISC</v>
       </c>
       <c r="C29" t="s">
@@ -1083,12 +1081,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>27</v>
       </c>
       <c r="B30" t="str">
-        <f>IF($A30="651","Barge1",IF($A30="101","Barge1",IF(A30="201","Barge 1",IF(A30="801","Barge 2",IF($A30="351", "Barge 2", IF($A30="151", "Barge 3",IF($A30="251","Barge 3",IF($A30="451", "Barge 4",IF($A30="551", "Barge 4",IF($A30="301","Barge 5",IF($A30="401","Barge 5",IF($A30="501","Barge 6",IF($A30="851","Barge 6",IF($A30="601","Barge 6",IF($A30="VC651","Barge1",IF($A30="VC101","Barge1",IF(A30="VC201","Barge 1",IF(A30="VC801","Barge 2",IF($A30="VC351", "Barge 2", IF($A30="VC151", "Barge 3",IF($A30="VC251","Barge 3",IF($A30="VC451", "Barge 4",IF($A30="VC551", "Barge 4",IF($A30="VC301","Barge 5",IF($A30="VC401","Barge 5",IF($A30="VC501","Barge 6",IF($A30="VC851","Barge 6",IF($A30="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>MISC</v>
       </c>
       <c r="C30" t="s">
@@ -1098,12 +1096,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>26</v>
       </c>
       <c r="B31" t="str">
-        <f>IF($A31="651","Barge1",IF($A31="101","Barge1",IF(A31="201","Barge 1",IF(A31="801","Barge 2",IF($A31="351", "Barge 2", IF($A31="151", "Barge 3",IF($A31="251","Barge 3",IF($A31="451", "Barge 4",IF($A31="551", "Barge 4",IF($A31="301","Barge 5",IF($A31="401","Barge 5",IF($A31="501","Barge 6",IF($A31="851","Barge 6",IF($A31="601","Barge 6",IF($A31="VC651","Barge1",IF($A31="VC101","Barge1",IF(A31="VC201","Barge 1",IF(A31="VC801","Barge 2",IF($A31="VC351", "Barge 2", IF($A31="VC151", "Barge 3",IF($A31="VC251","Barge 3",IF($A31="VC451", "Barge 4",IF($A31="VC551", "Barge 4",IF($A31="VC301","Barge 5",IF($A31="VC401","Barge 5",IF($A31="VC501","Barge 6",IF($A31="VC851","Barge 6",IF($A31="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>MISC</v>
       </c>
       <c r="C31" t="s">
@@ -1113,12 +1111,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>25</v>
       </c>
       <c r="B32" t="str">
-        <f>IF($A32="651","Barge1",IF($A32="101","Barge1",IF(A32="201","Barge 1",IF(A32="801","Barge 2",IF($A32="351", "Barge 2", IF($A32="151", "Barge 3",IF($A32="251","Barge 3",IF($A32="451", "Barge 4",IF($A32="551", "Barge 4",IF($A32="301","Barge 5",IF($A32="401","Barge 5",IF($A32="501","Barge 6",IF($A32="851","Barge 6",IF($A32="601","Barge 6",IF($A32="VC651","Barge1",IF($A32="VC101","Barge1",IF(A32="VC201","Barge 1",IF(A32="VC801","Barge 2",IF($A32="VC351", "Barge 2", IF($A32="VC151", "Barge 3",IF($A32="VC251","Barge 3",IF($A32="VC451", "Barge 4",IF($A32="VC551", "Barge 4",IF($A32="VC301","Barge 5",IF($A32="VC401","Barge 5",IF($A32="VC501","Barge 6",IF($A32="VC851","Barge 6",IF($A32="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>MISC</v>
       </c>
       <c r="C32" t="s">
@@ -1128,12 +1126,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>24</v>
       </c>
       <c r="B33" t="str">
-        <f>IF($A33="651","Barge1",IF($A33="101","Barge1",IF(A33="201","Barge 1",IF(A33="801","Barge 2",IF($A33="351", "Barge 2", IF($A33="151", "Barge 3",IF($A33="251","Barge 3",IF($A33="451", "Barge 4",IF($A33="551", "Barge 4",IF($A33="301","Barge 5",IF($A33="401","Barge 5",IF($A33="501","Barge 6",IF($A33="851","Barge 6",IF($A33="601","Barge 6",IF($A33="VC651","Barge1",IF($A33="VC101","Barge1",IF(A33="VC201","Barge 1",IF(A33="VC801","Barge 2",IF($A33="VC351", "Barge 2", IF($A33="VC151", "Barge 3",IF($A33="VC251","Barge 3",IF($A33="VC451", "Barge 4",IF($A33="VC551", "Barge 4",IF($A33="VC301","Barge 5",IF($A33="VC401","Barge 5",IF($A33="VC501","Barge 6",IF($A33="VC851","Barge 6",IF($A33="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="0"/>
         <v>MISC</v>
       </c>
       <c r="C33" t="s">
@@ -1143,12 +1141,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B34" t="str">
-        <f>IF($A34="651","Barge1",IF($A34="101","Barge1",IF(A34="201","Barge 1",IF(A34="801","Barge 2",IF($A34="351", "Barge 2", IF($A34="151", "Barge 3",IF($A34="251","Barge 3",IF($A34="451", "Barge 4",IF($A34="551", "Barge 4",IF($A34="301","Barge 5",IF($A34="401","Barge 5",IF($A34="501","Barge 6",IF($A34="851","Barge 6",IF($A34="601","Barge 6",IF($A34="VC651","Barge1",IF($A34="VC101","Barge1",IF(A34="VC201","Barge 1",IF(A34="VC801","Barge 2",IF($A34="VC351", "Barge 2", IF($A34="VC151", "Barge 3",IF($A34="VC251","Barge 3",IF($A34="VC451", "Barge 4",IF($A34="VC551", "Barge 4",IF($A34="VC301","Barge 5",IF($A34="VC401","Barge 5",IF($A34="VC501","Barge 6",IF($A34="VC851","Barge 6",IF($A34="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" ref="B34:B65" si="1">IF($A34="651","Barge1",IF($A34="101","Barge1",IF(A34="201","Barge 1",IF(A34="801","Barge 2",IF($A34="351", "Barge 2", IF($A34="151", "Barge 3",IF($A34="251","Barge 3",IF($A34="451", "Barge 4",IF($A34="551", "Barge 4",IF($A34="301","Barge 5",IF($A34="401","Barge 5",IF($A34="501","Barge 6",IF($A34="851","Barge 6",IF($A34="601","Barge 6",IF($A34="VC651","Barge1",IF($A34="VC101","Barge1",IF(A34="VC201","Barge 1",IF(A34="VC801","Barge 2",IF($A34="VC351", "Barge 2", IF($A34="VC151", "Barge 3",IF($A34="VC251","Barge 3",IF($A34="VC451", "Barge 4",IF($A34="VC551", "Barge 4",IF($A34="VC301","Barge 5",IF($A34="VC401","Barge 5",IF($A34="VC501","Barge 6",IF($A34="VC851","Barge 6",IF($A34="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
         <v>MISC</v>
       </c>
       <c r="C34" t="s">
@@ -1158,12 +1156,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>22</v>
       </c>
       <c r="B35" t="str">
-        <f>IF($A35="651","Barge1",IF($A35="101","Barge1",IF(A35="201","Barge 1",IF(A35="801","Barge 2",IF($A35="351", "Barge 2", IF($A35="151", "Barge 3",IF($A35="251","Barge 3",IF($A35="451", "Barge 4",IF($A35="551", "Barge 4",IF($A35="301","Barge 5",IF($A35="401","Barge 5",IF($A35="501","Barge 6",IF($A35="851","Barge 6",IF($A35="601","Barge 6",IF($A35="VC651","Barge1",IF($A35="VC101","Barge1",IF(A35="VC201","Barge 1",IF(A35="VC801","Barge 2",IF($A35="VC351", "Barge 2", IF($A35="VC151", "Barge 3",IF($A35="VC251","Barge 3",IF($A35="VC451", "Barge 4",IF($A35="VC551", "Barge 4",IF($A35="VC301","Barge 5",IF($A35="VC401","Barge 5",IF($A35="VC501","Barge 6",IF($A35="VC851","Barge 6",IF($A35="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C35" t="s">
@@ -1173,12 +1171,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>21</v>
       </c>
       <c r="B36" t="str">
-        <f>IF($A36="651","Barge1",IF($A36="101","Barge1",IF(A36="201","Barge 1",IF(A36="801","Barge 2",IF($A36="351", "Barge 2", IF($A36="151", "Barge 3",IF($A36="251","Barge 3",IF($A36="451", "Barge 4",IF($A36="551", "Barge 4",IF($A36="301","Barge 5",IF($A36="401","Barge 5",IF($A36="501","Barge 6",IF($A36="851","Barge 6",IF($A36="601","Barge 6",IF($A36="VC651","Barge1",IF($A36="VC101","Barge1",IF(A36="VC201","Barge 1",IF(A36="VC801","Barge 2",IF($A36="VC351", "Barge 2", IF($A36="VC151", "Barge 3",IF($A36="VC251","Barge 3",IF($A36="VC451", "Barge 4",IF($A36="VC551", "Barge 4",IF($A36="VC301","Barge 5",IF($A36="VC401","Barge 5",IF($A36="VC501","Barge 6",IF($A36="VC851","Barge 6",IF($A36="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C36" t="s">
@@ -1188,12 +1186,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>20</v>
       </c>
       <c r="B37" t="str">
-        <f>IF($A37="651","Barge1",IF($A37="101","Barge1",IF(A37="201","Barge 1",IF(A37="801","Barge 2",IF($A37="351", "Barge 2", IF($A37="151", "Barge 3",IF($A37="251","Barge 3",IF($A37="451", "Barge 4",IF($A37="551", "Barge 4",IF($A37="301","Barge 5",IF($A37="401","Barge 5",IF($A37="501","Barge 6",IF($A37="851","Barge 6",IF($A37="601","Barge 6",IF($A37="VC651","Barge1",IF($A37="VC101","Barge1",IF(A37="VC201","Barge 1",IF(A37="VC801","Barge 2",IF($A37="VC351", "Barge 2", IF($A37="VC151", "Barge 3",IF($A37="VC251","Barge 3",IF($A37="VC451", "Barge 4",IF($A37="VC551", "Barge 4",IF($A37="VC301","Barge 5",IF($A37="VC401","Barge 5",IF($A37="VC501","Barge 6",IF($A37="VC851","Barge 6",IF($A37="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C37" t="s">
@@ -1203,12 +1201,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B38" t="str">
-        <f>IF($A38="651","Barge1",IF($A38="101","Barge1",IF(A38="201","Barge 1",IF(A38="801","Barge 2",IF($A38="351", "Barge 2", IF($A38="151", "Barge 3",IF($A38="251","Barge 3",IF($A38="451", "Barge 4",IF($A38="551", "Barge 4",IF($A38="301","Barge 5",IF($A38="401","Barge 5",IF($A38="501","Barge 6",IF($A38="851","Barge 6",IF($A38="601","Barge 6",IF($A38="VC651","Barge1",IF($A38="VC101","Barge1",IF(A38="VC201","Barge 1",IF(A38="VC801","Barge 2",IF($A38="VC351", "Barge 2", IF($A38="VC151", "Barge 3",IF($A38="VC251","Barge 3",IF($A38="VC451", "Barge 4",IF($A38="VC551", "Barge 4",IF($A38="VC301","Barge 5",IF($A38="VC401","Barge 5",IF($A38="VC501","Barge 6",IF($A38="VC851","Barge 6",IF($A38="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C38" t="s">
@@ -1218,12 +1216,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>18</v>
       </c>
       <c r="B39" t="str">
-        <f>IF($A39="651","Barge1",IF($A39="101","Barge1",IF(A39="201","Barge 1",IF(A39="801","Barge 2",IF($A39="351", "Barge 2", IF($A39="151", "Barge 3",IF($A39="251","Barge 3",IF($A39="451", "Barge 4",IF($A39="551", "Barge 4",IF($A39="301","Barge 5",IF($A39="401","Barge 5",IF($A39="501","Barge 6",IF($A39="851","Barge 6",IF($A39="601","Barge 6",IF($A39="VC651","Barge1",IF($A39="VC101","Barge1",IF(A39="VC201","Barge 1",IF(A39="VC801","Barge 2",IF($A39="VC351", "Barge 2", IF($A39="VC151", "Barge 3",IF($A39="VC251","Barge 3",IF($A39="VC451", "Barge 4",IF($A39="VC551", "Barge 4",IF($A39="VC301","Barge 5",IF($A39="VC401","Barge 5",IF($A39="VC501","Barge 6",IF($A39="VC851","Barge 6",IF($A39="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C39" t="s">
@@ -1233,12 +1231,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>17</v>
       </c>
       <c r="B40" t="str">
-        <f>IF($A40="651","Barge1",IF($A40="101","Barge1",IF(A40="201","Barge 1",IF(A40="801","Barge 2",IF($A40="351", "Barge 2", IF($A40="151", "Barge 3",IF($A40="251","Barge 3",IF($A40="451", "Barge 4",IF($A40="551", "Barge 4",IF($A40="301","Barge 5",IF($A40="401","Barge 5",IF($A40="501","Barge 6",IF($A40="851","Barge 6",IF($A40="601","Barge 6",IF($A40="VC651","Barge1",IF($A40="VC101","Barge1",IF(A40="VC201","Barge 1",IF(A40="VC801","Barge 2",IF($A40="VC351", "Barge 2", IF($A40="VC151", "Barge 3",IF($A40="VC251","Barge 3",IF($A40="VC451", "Barge 4",IF($A40="VC551", "Barge 4",IF($A40="VC301","Barge 5",IF($A40="VC401","Barge 5",IF($A40="VC501","Barge 6",IF($A40="VC851","Barge 6",IF($A40="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C40" t="s">
@@ -1248,12 +1246,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B41" t="str">
-        <f>IF($A41="651","Barge1",IF($A41="101","Barge1",IF(A41="201","Barge 1",IF(A41="801","Barge 2",IF($A41="351", "Barge 2", IF($A41="151", "Barge 3",IF($A41="251","Barge 3",IF($A41="451", "Barge 4",IF($A41="551", "Barge 4",IF($A41="301","Barge 5",IF($A41="401","Barge 5",IF($A41="501","Barge 6",IF($A41="851","Barge 6",IF($A41="601","Barge 6",IF($A41="VC651","Barge1",IF($A41="VC101","Barge1",IF(A41="VC201","Barge 1",IF(A41="VC801","Barge 2",IF($A41="VC351", "Barge 2", IF($A41="VC151", "Barge 3",IF($A41="VC251","Barge 3",IF($A41="VC451", "Barge 4",IF($A41="VC551", "Barge 4",IF($A41="VC301","Barge 5",IF($A41="VC401","Barge 5",IF($A41="VC501","Barge 6",IF($A41="VC851","Barge 6",IF($A41="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C41" t="s">
@@ -1263,12 +1261,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B42" t="str">
-        <f>IF($A42="651","Barge1",IF($A42="101","Barge1",IF(A42="201","Barge 1",IF(A42="801","Barge 2",IF($A42="351", "Barge 2", IF($A42="151", "Barge 3",IF($A42="251","Barge 3",IF($A42="451", "Barge 4",IF($A42="551", "Barge 4",IF($A42="301","Barge 5",IF($A42="401","Barge 5",IF($A42="501","Barge 6",IF($A42="851","Barge 6",IF($A42="601","Barge 6",IF($A42="VC651","Barge1",IF($A42="VC101","Barge1",IF(A42="VC201","Barge 1",IF(A42="VC801","Barge 2",IF($A42="VC351", "Barge 2", IF($A42="VC151", "Barge 3",IF($A42="VC251","Barge 3",IF($A42="VC451", "Barge 4",IF($A42="VC551", "Barge 4",IF($A42="VC301","Barge 5",IF($A42="VC401","Barge 5",IF($A42="VC501","Barge 6",IF($A42="VC851","Barge 6",IF($A42="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C42" t="s">
@@ -1278,12 +1276,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>14</v>
       </c>
       <c r="B43" t="str">
-        <f>IF($A43="651","Barge1",IF($A43="101","Barge1",IF(A43="201","Barge 1",IF(A43="801","Barge 2",IF($A43="351", "Barge 2", IF($A43="151", "Barge 3",IF($A43="251","Barge 3",IF($A43="451", "Barge 4",IF($A43="551", "Barge 4",IF($A43="301","Barge 5",IF($A43="401","Barge 5",IF($A43="501","Barge 6",IF($A43="851","Barge 6",IF($A43="601","Barge 6",IF($A43="VC651","Barge1",IF($A43="VC101","Barge1",IF(A43="VC201","Barge 1",IF(A43="VC801","Barge 2",IF($A43="VC351", "Barge 2", IF($A43="VC151", "Barge 3",IF($A43="VC251","Barge 3",IF($A43="VC451", "Barge 4",IF($A43="VC551", "Barge 4",IF($A43="VC301","Barge 5",IF($A43="VC401","Barge 5",IF($A43="VC501","Barge 6",IF($A43="VC851","Barge 6",IF($A43="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C43" t="s">
@@ -1293,12 +1291,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>13</v>
       </c>
       <c r="B44" t="str">
-        <f>IF($A44="651","Barge1",IF($A44="101","Barge1",IF(A44="201","Barge 1",IF(A44="801","Barge 2",IF($A44="351", "Barge 2", IF($A44="151", "Barge 3",IF($A44="251","Barge 3",IF($A44="451", "Barge 4",IF($A44="551", "Barge 4",IF($A44="301","Barge 5",IF($A44="401","Barge 5",IF($A44="501","Barge 6",IF($A44="851","Barge 6",IF($A44="601","Barge 6",IF($A44="VC651","Barge1",IF($A44="VC101","Barge1",IF(A44="VC201","Barge 1",IF(A44="VC801","Barge 2",IF($A44="VC351", "Barge 2", IF($A44="VC151", "Barge 3",IF($A44="VC251","Barge 3",IF($A44="VC451", "Barge 4",IF($A44="VC551", "Barge 4",IF($A44="VC301","Barge 5",IF($A44="VC401","Barge 5",IF($A44="VC501","Barge 6",IF($A44="VC851","Barge 6",IF($A44="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C44" t="s">
@@ -1308,12 +1306,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>12</v>
       </c>
       <c r="B45" t="str">
-        <f>IF($A45="651","Barge1",IF($A45="101","Barge1",IF(A45="201","Barge 1",IF(A45="801","Barge 2",IF($A45="351", "Barge 2", IF($A45="151", "Barge 3",IF($A45="251","Barge 3",IF($A45="451", "Barge 4",IF($A45="551", "Barge 4",IF($A45="301","Barge 5",IF($A45="401","Barge 5",IF($A45="501","Barge 6",IF($A45="851","Barge 6",IF($A45="601","Barge 6",IF($A45="VC651","Barge1",IF($A45="VC101","Barge1",IF(A45="VC201","Barge 1",IF(A45="VC801","Barge 2",IF($A45="VC351", "Barge 2", IF($A45="VC151", "Barge 3",IF($A45="VC251","Barge 3",IF($A45="VC451", "Barge 4",IF($A45="VC551", "Barge 4",IF($A45="VC301","Barge 5",IF($A45="VC401","Barge 5",IF($A45="VC501","Barge 6",IF($A45="VC851","Barge 6",IF($A45="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C45" t="s">
@@ -1323,12 +1321,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>11</v>
       </c>
       <c r="B46" t="str">
-        <f>IF($A46="651","Barge1",IF($A46="101","Barge1",IF(A46="201","Barge 1",IF(A46="801","Barge 2",IF($A46="351", "Barge 2", IF($A46="151", "Barge 3",IF($A46="251","Barge 3",IF($A46="451", "Barge 4",IF($A46="551", "Barge 4",IF($A46="301","Barge 5",IF($A46="401","Barge 5",IF($A46="501","Barge 6",IF($A46="851","Barge 6",IF($A46="601","Barge 6",IF($A46="VC651","Barge1",IF($A46="VC101","Barge1",IF(A46="VC201","Barge 1",IF(A46="VC801","Barge 2",IF($A46="VC351", "Barge 2", IF($A46="VC151", "Barge 3",IF($A46="VC251","Barge 3",IF($A46="VC451", "Barge 4",IF($A46="VC551", "Barge 4",IF($A46="VC301","Barge 5",IF($A46="VC401","Barge 5",IF($A46="VC501","Barge 6",IF($A46="VC851","Barge 6",IF($A46="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C46" t="s">
@@ -1338,12 +1336,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>10</v>
       </c>
       <c r="B47" t="str">
-        <f>IF($A47="651","Barge1",IF($A47="101","Barge1",IF(A47="201","Barge 1",IF(A47="801","Barge 2",IF($A47="351", "Barge 2", IF($A47="151", "Barge 3",IF($A47="251","Barge 3",IF($A47="451", "Barge 4",IF($A47="551", "Barge 4",IF($A47="301","Barge 5",IF($A47="401","Barge 5",IF($A47="501","Barge 6",IF($A47="851","Barge 6",IF($A47="601","Barge 6",IF($A47="VC651","Barge1",IF($A47="VC101","Barge1",IF(A47="VC201","Barge 1",IF(A47="VC801","Barge 2",IF($A47="VC351", "Barge 2", IF($A47="VC151", "Barge 3",IF($A47="VC251","Barge 3",IF($A47="VC451", "Barge 4",IF($A47="VC551", "Barge 4",IF($A47="VC301","Barge 5",IF($A47="VC401","Barge 5",IF($A47="VC501","Barge 6",IF($A47="VC851","Barge 6",IF($A47="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C47" t="s">
@@ -1353,12 +1351,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>9</v>
       </c>
       <c r="B48" t="str">
-        <f>IF($A48="651","Barge1",IF($A48="101","Barge1",IF(A48="201","Barge 1",IF(A48="801","Barge 2",IF($A48="351", "Barge 2", IF($A48="151", "Barge 3",IF($A48="251","Barge 3",IF($A48="451", "Barge 4",IF($A48="551", "Barge 4",IF($A48="301","Barge 5",IF($A48="401","Barge 5",IF($A48="501","Barge 6",IF($A48="851","Barge 6",IF($A48="601","Barge 6",IF($A48="VC651","Barge1",IF($A48="VC101","Barge1",IF(A48="VC201","Barge 1",IF(A48="VC801","Barge 2",IF($A48="VC351", "Barge 2", IF($A48="VC151", "Barge 3",IF($A48="VC251","Barge 3",IF($A48="VC451", "Barge 4",IF($A48="VC551", "Barge 4",IF($A48="VC301","Barge 5",IF($A48="VC401","Barge 5",IF($A48="VC501","Barge 6",IF($A48="VC851","Barge 6",IF($A48="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C48" t="s">
@@ -1368,12 +1366,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>8</v>
       </c>
       <c r="B49" t="str">
-        <f>IF($A49="651","Barge1",IF($A49="101","Barge1",IF(A49="201","Barge 1",IF(A49="801","Barge 2",IF($A49="351", "Barge 2", IF($A49="151", "Barge 3",IF($A49="251","Barge 3",IF($A49="451", "Barge 4",IF($A49="551", "Barge 4",IF($A49="301","Barge 5",IF($A49="401","Barge 5",IF($A49="501","Barge 6",IF($A49="851","Barge 6",IF($A49="601","Barge 6",IF($A49="VC651","Barge1",IF($A49="VC101","Barge1",IF(A49="VC201","Barge 1",IF(A49="VC801","Barge 2",IF($A49="VC351", "Barge 2", IF($A49="VC151", "Barge 3",IF($A49="VC251","Barge 3",IF($A49="VC451", "Barge 4",IF($A49="VC551", "Barge 4",IF($A49="VC301","Barge 5",IF($A49="VC401","Barge 5",IF($A49="VC501","Barge 6",IF($A49="VC851","Barge 6",IF($A49="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C49" t="s">
@@ -1383,12 +1381,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>7</v>
       </c>
       <c r="B50" t="str">
-        <f>IF($A50="651","Barge1",IF($A50="101","Barge1",IF(A50="201","Barge 1",IF(A50="801","Barge 2",IF($A50="351", "Barge 2", IF($A50="151", "Barge 3",IF($A50="251","Barge 3",IF($A50="451", "Barge 4",IF($A50="551", "Barge 4",IF($A50="301","Barge 5",IF($A50="401","Barge 5",IF($A50="501","Barge 6",IF($A50="851","Barge 6",IF($A50="601","Barge 6",IF($A50="VC651","Barge1",IF($A50="VC101","Barge1",IF(A50="VC201","Barge 1",IF(A50="VC801","Barge 2",IF($A50="VC351", "Barge 2", IF($A50="VC151", "Barge 3",IF($A50="VC251","Barge 3",IF($A50="VC451", "Barge 4",IF($A50="VC551", "Barge 4",IF($A50="VC301","Barge 5",IF($A50="VC401","Barge 5",IF($A50="VC501","Barge 6",IF($A50="VC851","Barge 6",IF($A50="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C50" t="s">
@@ -1398,12 +1396,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>6</v>
       </c>
       <c r="B51" t="str">
-        <f>IF($A51="651","Barge1",IF($A51="101","Barge1",IF(A51="201","Barge 1",IF(A51="801","Barge 2",IF($A51="351", "Barge 2", IF($A51="151", "Barge 3",IF($A51="251","Barge 3",IF($A51="451", "Barge 4",IF($A51="551", "Barge 4",IF($A51="301","Barge 5",IF($A51="401","Barge 5",IF($A51="501","Barge 6",IF($A51="851","Barge 6",IF($A51="601","Barge 6",IF($A51="VC651","Barge1",IF($A51="VC101","Barge1",IF(A51="VC201","Barge 1",IF(A51="VC801","Barge 2",IF($A51="VC351", "Barge 2", IF($A51="VC151", "Barge 3",IF($A51="VC251","Barge 3",IF($A51="VC451", "Barge 4",IF($A51="VC551", "Barge 4",IF($A51="VC301","Barge 5",IF($A51="VC401","Barge 5",IF($A51="VC501","Barge 6",IF($A51="VC851","Barge 6",IF($A51="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C51" t="s">
@@ -1413,12 +1411,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>5</v>
       </c>
       <c r="B52" t="str">
-        <f>IF($A52="651","Barge1",IF($A52="101","Barge1",IF(A52="201","Barge 1",IF(A52="801","Barge 2",IF($A52="351", "Barge 2", IF($A52="151", "Barge 3",IF($A52="251","Barge 3",IF($A52="451", "Barge 4",IF($A52="551", "Barge 4",IF($A52="301","Barge 5",IF($A52="401","Barge 5",IF($A52="501","Barge 6",IF($A52="851","Barge 6",IF($A52="601","Barge 6",IF($A52="VC651","Barge1",IF($A52="VC101","Barge1",IF(A52="VC201","Barge 1",IF(A52="VC801","Barge 2",IF($A52="VC351", "Barge 2", IF($A52="VC151", "Barge 3",IF($A52="VC251","Barge 3",IF($A52="VC451", "Barge 4",IF($A52="VC551", "Barge 4",IF($A52="VC301","Barge 5",IF($A52="VC401","Barge 5",IF($A52="VC501","Barge 6",IF($A52="VC851","Barge 6",IF($A52="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C52" t="s">
@@ -1428,12 +1426,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>4</v>
       </c>
       <c r="B53" t="str">
-        <f>IF($A53="651","Barge1",IF($A53="101","Barge1",IF(A53="201","Barge 1",IF(A53="801","Barge 2",IF($A53="351", "Barge 2", IF($A53="151", "Barge 3",IF($A53="251","Barge 3",IF($A53="451", "Barge 4",IF($A53="551", "Barge 4",IF($A53="301","Barge 5",IF($A53="401","Barge 5",IF($A53="501","Barge 6",IF($A53="851","Barge 6",IF($A53="601","Barge 6",IF($A53="VC651","Barge1",IF($A53="VC101","Barge1",IF(A53="VC201","Barge 1",IF(A53="VC801","Barge 2",IF($A53="VC351", "Barge 2", IF($A53="VC151", "Barge 3",IF($A53="VC251","Barge 3",IF($A53="VC451", "Barge 4",IF($A53="VC551", "Barge 4",IF($A53="VC301","Barge 5",IF($A53="VC401","Barge 5",IF($A53="VC501","Barge 6",IF($A53="VC851","Barge 6",IF($A53="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C53" t="s">
@@ -1443,12 +1441,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>3</v>
       </c>
       <c r="B54" t="str">
-        <f>IF($A54="651","Barge1",IF($A54="101","Barge1",IF(A54="201","Barge 1",IF(A54="801","Barge 2",IF($A54="351", "Barge 2", IF($A54="151", "Barge 3",IF($A54="251","Barge 3",IF($A54="451", "Barge 4",IF($A54="551", "Barge 4",IF($A54="301","Barge 5",IF($A54="401","Barge 5",IF($A54="501","Barge 6",IF($A54="851","Barge 6",IF($A54="601","Barge 6",IF($A54="VC651","Barge1",IF($A54="VC101","Barge1",IF(A54="VC201","Barge 1",IF(A54="VC801","Barge 2",IF($A54="VC351", "Barge 2", IF($A54="VC151", "Barge 3",IF($A54="VC251","Barge 3",IF($A54="VC451", "Barge 4",IF($A54="VC551", "Barge 4",IF($A54="VC301","Barge 5",IF($A54="VC401","Barge 5",IF($A54="VC501","Barge 6",IF($A54="VC851","Barge 6",IF($A54="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C54" t="s">
@@ -1458,12 +1456,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>2</v>
       </c>
       <c r="B55" t="str">
-        <f>IF($A55="651","Barge1",IF($A55="101","Barge1",IF(A55="201","Barge 1",IF(A55="801","Barge 2",IF($A55="351", "Barge 2", IF($A55="151", "Barge 3",IF($A55="251","Barge 3",IF($A55="451", "Barge 4",IF($A55="551", "Barge 4",IF($A55="301","Barge 5",IF($A55="401","Barge 5",IF($A55="501","Barge 6",IF($A55="851","Barge 6",IF($A55="601","Barge 6",IF($A55="VC651","Barge1",IF($A55="VC101","Barge1",IF(A55="VC201","Barge 1",IF(A55="VC801","Barge 2",IF($A55="VC351", "Barge 2", IF($A55="VC151", "Barge 3",IF($A55="VC251","Barge 3",IF($A55="VC451", "Barge 4",IF($A55="VC551", "Barge 4",IF($A55="VC301","Barge 5",IF($A55="VC401","Barge 5",IF($A55="VC501","Barge 6",IF($A55="VC851","Barge 6",IF($A55="VC601","Barge 6","MISC"))))))))))))))))))))))))))))</f>
+        <f t="shared" si="1"/>
         <v>MISC</v>
       </c>
       <c r="C55" t="s">
@@ -1474,6 +1472,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <conditionalFormatting sqref="A2:A55">
     <cfRule type="containsText" dxfId="1" priority="1" operator="containsText" text="651, 101, 251, 151, 201">
       <formula>NOT(ISERROR(SEARCH("651, 101, 251, 151, 201",A2)))</formula>
@@ -1483,5 +1482,60 @@
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="360" verticalDpi="360" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8EF82B4A-4329-495B-9E1C-88F6B221F250}">
+  <dimension ref="A1:A8"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="13.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A5" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="A8" t="s">
+        <v>73</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>